<commit_message>
update read-excel examples and data files
</commit_message>
<xml_diff>
--- a/data/lab_results.xlsx
+++ b/data/lab_results.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Dissolution" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Titration" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Calibration" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Weights (missing)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2403,4 +2404,350 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>tablet_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>weight_mg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>506.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>498.1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>503.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>502.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>500.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>506.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>507.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>498.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>504.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>508.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>493.2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>498.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>501.7</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>500.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>490.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>491.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>500.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>500.8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>506.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>